<commit_message>
Revamp Jamali dashboard and audit XLSX fixtures
</commit_message>
<xml_diff>
--- a/samples/ss_cwd_ingest.xlsx
+++ b/samples/ss_cwd_ingest.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -501,6 +501,10 @@
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -559,6 +563,26 @@
           <t>Wilayah</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Jumlah Trafo</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Jumlah Kapasitor</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Catatan Simbol</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -803,7 +827,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -819,6 +843,12 @@
         <is>
           <t>Banten</t>
         </is>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -841,7 +871,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -857,6 +887,12 @@
         <is>
           <t>Banten</t>
         </is>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -879,7 +915,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -894,6 +930,17 @@
       <c r="K9" t="inlineStr">
         <is>
           <t>Banten</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>3</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>SLD PLN Cawang-Depok 2.7</t>
         </is>
       </c>
     </row>
@@ -917,7 +964,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -933,6 +980,12 @@
         <is>
           <t>Banten</t>
         </is>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -955,7 +1008,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -971,6 +1024,12 @@
         <is>
           <t>Banten</t>
         </is>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -993,7 +1052,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1009,6 +1068,12 @@
         <is>
           <t>Banten</t>
         </is>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1031,7 +1096,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1050,6 +1115,12 @@
         <is>
           <t>Banten</t>
         </is>
+      </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1072,7 +1143,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1088,6 +1159,12 @@
         <is>
           <t>Banten</t>
         </is>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1110,7 +1187,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1126,6 +1203,12 @@
         <is>
           <t>Banten</t>
         </is>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1148,7 +1231,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1167,6 +1250,12 @@
         <is>
           <t>Banten</t>
         </is>
+      </c>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1180,7 +1269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1198,6 +1287,7 @@
     <col width="19" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1276,6 +1366,11 @@
           <t>Tier Ke</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Single Phi</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1322,6 +1417,11 @@
           <t>Banten</t>
         </is>
       </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1365,6 +1465,11 @@
           <t>Banten</t>
         </is>
       </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1408,6 +1513,11 @@
           <t>Banten</t>
         </is>
       </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1451,6 +1561,11 @@
           <t>Banten</t>
         </is>
       </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1494,6 +1609,11 @@
           <t>Banten</t>
         </is>
       </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1537,6 +1657,11 @@
           <t>Banten</t>
         </is>
       </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1580,6 +1705,11 @@
           <t>Banten</t>
         </is>
       </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1623,6 +1753,11 @@
           <t>Banten</t>
         </is>
       </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1666,6 +1801,11 @@
           <t>Banten</t>
         </is>
       </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1707,6 +1847,11 @@
       <c r="M11" t="inlineStr">
         <is>
           <t>Banten</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1729,8 +1874,10 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1761,12 +1908,22 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Jumlah Sirkit</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Status Operasi</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>No Kerawanan</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Sudut Pandang</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1951,10 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
@@ -1824,7 +1984,10 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
@@ -1854,7 +2017,10 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>

</xml_diff>